<commit_message>
idiom: create bar graph
</commit_message>
<xml_diff>
--- a/data/m_pa.xlsx
+++ b/data/m_pa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\_MONASH_UNI\_Y3S1\FIT3179\DV2_repo\FIT3179_DV2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{883D73C8-9AEA-4BA6-B664-E15A98DE6E42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BA640DC-087E-466A-B381-0AE091C8BC3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -5573,6 +5573,7 @@
     <col min="2" max="2" width="19.88671875" customWidth="1"/>
     <col min="3" max="3" width="27.109375" customWidth="1"/>
     <col min="4" max="5" width="30.5546875" customWidth="1"/>
+    <col min="8" max="8" width="18.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
feature: create chart for ibra bioregion
</commit_message>
<xml_diff>
--- a/data/m_pa.xlsx
+++ b/data/m_pa.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\_MONASH_UNI\_Y3S1\FIT3179\DV2_repo\FIT3179_DV2\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BA640DC-087E-466A-B381-0AE091C8BC3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C9A110B-730E-4704-9D25-39D1E9DF573D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$D$41</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -65,9 +65,6 @@
     <t>Queensland</t>
   </si>
   <si>
-    <t>Nothern Territory</t>
-  </si>
-  <si>
     <t>Protected Area (ha)</t>
   </si>
   <si>
@@ -81,6 +78,9 @@
   </si>
   <si>
     <t>Commonwealth</t>
+  </si>
+  <si>
+    <t>Northern Territory</t>
   </si>
 </sst>
 </file>
@@ -5584,16 +5584,16 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -5620,7 +5620,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B3" s="3">
         <v>2016</v>
@@ -5774,7 +5774,7 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B10" s="3">
         <v>2018</v>
@@ -5928,7 +5928,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B17" s="3">
         <v>2020</v>
@@ -6082,7 +6082,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B24" s="3">
         <v>2022</v>
@@ -6236,7 +6236,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B31" s="3">
         <v>2024</v>
@@ -6368,7 +6368,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B37" s="3">
         <v>2016</v>
@@ -6390,7 +6390,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B38" s="3">
         <v>2018</v>
@@ -6412,7 +6412,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B39" s="3">
         <v>2020</v>
@@ -6434,7 +6434,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B40" s="3">
         <v>2022</v>
@@ -6456,7 +6456,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B41" s="3">
         <v>2024</v>
@@ -6480,7 +6480,7 @@
       <c r="D42" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D36" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:D41" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>